<commit_message>
Corrections in number of symbols
</commit_message>
<xml_diff>
--- a/reference_keys/KEY_PlayInterventionTraining_1.xlsx
+++ b/reference_keys/KEY_PlayInterventionTraining_1.xlsx
@@ -1421,7 +1421,7 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47">
@@ -1681,7 +1681,7 @@
         </is>
       </c>
       <c r="J59" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60">

</xml_diff>